<commit_message>
Update Q4 audit planning artifacts
</commit_message>
<xml_diff>
--- a/01-Planejamento/03-Estrategia_e_Plano/04-Matriz_Planejamento/matriz_verificaca_evidencias.xlsx
+++ b/01-Planejamento/03-Estrategia_e_Plano/04-Matriz_Planejamento/matriz_verificaca_evidencias.xlsx
@@ -9,10 +9,14 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q1_Checklists" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q2_Checklists" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q3_Checklists" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q4_Checklists" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Q1_Checklists'!$A$1:$F$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Q2_Checklists'!$A$1:$F$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Q3_Checklists'!$A$1:$F$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Q4_Checklists'!$A$1:$F$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1399,4 +1403,987 @@
   <autoFilter ref="A1:F8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="78" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="56" customWidth="1" min="5" max="5"/>
+    <col width="130" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>id_avaliacao</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>questao_auditoria</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>situacao_encontrada</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>item_evidencia</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>descricao_avaliacao</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>prompt_checklist</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="210" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Q3-S3.2-q2703evi</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Q3 - Capacidade Institucional de TIC e Segurança da Informação</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>S3.2 - A organização não definiu o quantitativo necessário de pessoal de TIC e segurança da informação.</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>q2703evi</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Verificar se a evidência comprova definição documentada do quantitativo necessário de pessoal de TIC/SI com base em critérios ou procedimentos técnicos.</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Você é avaliador de evidências da Fiscalização TCE-RJ nº 18/2026 - iGovTI 2026. Analise exclusivamente a evidência anexada ao item indicado. Não busque informações externas, não presuma fatos não documentados e não utilize conhecimento fora da evidência fornecida.
+ID da avaliação: Q3-S3.2-q2703evi.
+Objetivo da avaliação: verificar se a evidência comprova definição documentada do quantitativo necessário de pessoal de TIC e segurança da informação com base em critérios ou procedimentos técnicos.
+Contexto da situação encontrada: S3.2 - A organização não definiu o quantitativo necessário de pessoal de TIC e segurança da informação.
+Item de evidência avaliado: q2703evi.
+Evidência esperada no questionário: política ou metodologia de dimensionamento; estudos ou relatórios técnicos; definição documentada do quantitativo necessário; critérios utilizados, como serviços, sistemas, demanda, riscos ou complexidade; revisões periódicas; planos de provimento; ou outras evidências cabíveis, indicando a abrangência na organização.
+Critérios da matriz aplicáveis: C2 - COBIT 2019 APO07.01; C5 - COBIT 2019 APO07.05; C9 - ABNT NBR ISO/IEC 27001:2022, cláusulas 5.3 e 7.2.
+Checklist obrigatório:
+1. Identifique o tipo documental apresentado e se ele possui caráter formal, técnico ou institucional.
+2. Verifique se a evidência se refere à organização auditada e ao período ou contexto avaliado.
+3. Verifique se há definição do quantitativo necessário de pessoal de TIC e de segurança da informação, e não apenas relação do quadro atual.
+4. Verifique se o dimensionamento está baseado em critérios ou procedimentos técnicos, como porte, serviços, sistemas, demandas, riscos, contratos ou complexidade.
+5. Verifique se a evidência indica abrangência, premissas, unidade responsável ou processo de revisão do dimensionamento.
+6. Verifique se a evidência é compatível com as respostas declaradas em q2703ext[B] e q2703ext[C].
+7. Decida se a evidência comprova, de forma suficiente, a definição documentada do quantitativo necessário de pessoal de TIC/SI.
+Ao aplicar o checklist, considere a evidência como um target binário para a regra de identificação da situação encontrada. O resultado "Não conforme" será usado pela matriz como indicativo de evidência inexistente, incompatível ou insuficiente para comprovar a prática avaliada.
+Contrato de saída obrigatório:
+Responda exclusivamente em JSON válido, sem texto fora do JSON, com os campos:
+{
+  "id_avaliacao": "Q3-S3.2-q2703evi",
+  "resultado": "Conforme" ou "Não conforme",
+  "justificativa_sintetica": "&lt;fundamento objetivo da decisão&gt;",
+  "elementos_comprovados": ["&lt;elementos relevantes comprovados&gt;"],
+  "lacunas": ["&lt;elementos obrigatórios ausentes ou insuficientes&gt;"],
+  "inconsistencias": ["&lt;incompatibilidades entre evidência, resposta declarada ou escopo&gt;"]
+}
+Regra de decisão binária:
+- Retorne "Conforme" somente quando a evidência for existente, compatível e suficiente para comprovar todos os elementos essenciais da avaliação descrita.
+- Retorne "Não conforme" quando a evidência for inexistente, ilegível, incompatível, desatualizada, meramente declaratória sem comprovação documental suficiente, ou quando faltar qualquer elemento essencial da avaliação.
+- Não use classificações intermediárias, como parcialmente conforme, parcialmente suficiente ou inconclusivo. Em caso de dúvida relevante, retorne "Não conforme" e descreva a lacuna.
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="210" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Q3-S3.4-q2701evi</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Q3 - Capacidade Institucional de TIC e Segurança da Informação</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>S3.4 - Perfis profissionais de TIC e segurança da informação inexistentes, insuficientes ou não utilizados na escolha de gestores.</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>q2701evi</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Verificar se a evidência comprova perfis profissionais definidos para gestores de TIC e segurança da informação.</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Você é avaliador de evidências da Fiscalização TCE-RJ nº 18/2026 - iGovTI 2026. Analise exclusivamente a evidência anexada ao item indicado. Não busque informações externas, não presuma fatos não documentados e não utilize conhecimento fora da evidência fornecida.
+ID da avaliação: Q3-S3.4-q2701evi.
+Objetivo da avaliação: verificar se a evidência comprova perfis profissionais definidos e documentados para gestores de TIC e segurança da informação.
+Contexto da situação encontrada: S3.4 - Perfis profissionais de TIC e segurança da informação inexistentes, insuficientes ou não utilizados na escolha de gestores.
+Item de evidência avaliado: q2701evi.
+Evidência esperada no questionário: normativos ou documentos com atribuições e competências; descrições de cargos ou funções; matrizes de competências; registros de revisão periódica; publicações em portal institucional ou transparência ativa; atos de designação; ou outras evidências cabíveis, indicando a abrangência na organização.
+Critérios da matriz aplicáveis: C1 - COBIT 2019 APO01.05; C4 - COBIT 2019 APO07.03; C9 - ABNT NBR ISO/IEC 27001:2022, cláusulas 5.3 e 7.2; C10 - ABNT NBR ISO/IEC 27002:2022, controles 5.2 e 6.3.
+Checklist obrigatório:
+1. Identifique o tipo documental apresentado e se ele possui caráter formal ou institucional.
+2. Verifique se o documento define responsabilidades e atribuições de gestores de TIC ou segurança da informação.
+3. Verifique se o documento relaciona competências, habilidades, experiência ou requisitos mínimos esperados para os gestores.
+4. Verifique se os perfis são aplicáveis à organização auditada e às funções de gestão avaliadas.
+5. Verifique se há indício de publicação, comunicação, revisão periódica ou uso institucional dos perfis.
+6. Verifique se a evidência é compatível com as respostas declaradas em q2701ext[A] e q2701ext[C].
+7. Decida se a evidência comprova, de forma suficiente, perfis profissionais definidos para gestores de TIC/SI.
+Ao aplicar o checklist, considere a evidência como um target binário para a regra de identificação da situação encontrada. O resultado "Não conforme" será usado pela matriz como indicativo de evidência inexistente, incompatível ou insuficiente para comprovar a prática avaliada.
+Contrato de saída obrigatório:
+Responda exclusivamente em JSON válido, sem texto fora do JSON, com os campos:
+{
+  "id_avaliacao": "Q3-S3.4-q2701evi",
+  "resultado": "Conforme" ou "Não conforme",
+  "justificativa_sintetica": "&lt;fundamento objetivo da decisão&gt;",
+  "elementos_comprovados": ["&lt;elementos relevantes comprovados&gt;"],
+  "lacunas": ["&lt;elementos obrigatórios ausentes ou insuficientes&gt;"],
+  "inconsistencias": ["&lt;incompatibilidades entre evidência, resposta declarada ou escopo&gt;"]
+}
+Regra de decisão binária:
+- Retorne "Conforme" somente quando a evidência for existente, compatível e suficiente para comprovar todos os elementos essenciais da avaliação descrita.
+- Retorne "Não conforme" quando a evidência for inexistente, ilegível, incompatível, desatualizada, meramente declaratória sem comprovação documental suficiente, ou quando faltar qualquer elemento essencial da avaliação.
+- Não use classificações intermediárias, como parcialmente conforme, parcialmente suficiente ou inconclusivo. Em caso de dúvida relevante, retorne "Não conforme" e descreva a lacuna.
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="210" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Q3-S3.4-q2702evi</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Q3 - Capacidade Institucional de TIC e Segurança da Informação</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>S3.4 - Perfis profissionais de TIC e segurança da informação inexistentes, insuficientes ou não utilizados na escolha de gestores.</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>q2702evi</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Verificar se a evidência comprova perfis profissionais definidos para colaboradores de TIC e segurança da informação.</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Você é avaliador de evidências da Fiscalização TCE-RJ nº 18/2026 - iGovTI 2026. Analise exclusivamente a evidência anexada ao item indicado. Não busque informações externas, não presuma fatos não documentados e não utilize conhecimento fora da evidência fornecida.
+ID da avaliação: Q3-S3.4-q2702evi.
+Objetivo da avaliação: verificar se a evidência comprova perfis profissionais definidos e documentados para colaboradores de TIC e segurança da informação.
+Contexto da situação encontrada: S3.4 - Perfis profissionais de TIC e segurança da informação inexistentes, insuficientes ou não utilizados na escolha de gestores.
+Item de evidência avaliado: q2702evi.
+Evidência esperada no questionário: descrições de cargos ou funções; matrizes de competências; normativos com atribuições e responsabilidades; registros de revisão periódica; publicações em portal institucional ou mecanismos de transparência; planos de capacitação relacionados; ou outras evidências cabíveis, indicando a abrangência na organização.
+Critérios da matriz aplicáveis: C1 - COBIT 2019 APO01.05; C4 - COBIT 2019 APO07.03; C9 - ABNT NBR ISO/IEC 27001:2022, cláusulas 5.3 e 7.2; C10 - ABNT NBR ISO/IEC 27002:2022, controles 5.2 e 6.3.
+Checklist obrigatório:
+1. Identifique o tipo documental apresentado e se ele possui caráter formal ou institucional.
+2. Verifique se o documento define responsabilidades e atribuições de colaboradores, ocupações ou grupos de ocupações de TIC/SI.
+3. Verifique se o documento relaciona competências, habilidades, experiência ou requisitos mínimos esperados para os colaboradores.
+4. Verifique se os perfis abrangem funções essenciais de TIC, segurança da informação ou sustentação tecnológica compatíveis com o escopo da organização.
+5. Verifique se há indício de publicação, comunicação, revisão periódica ou uso institucional dos perfis.
+6. Verifique se a evidência é compatível com as respostas declaradas em q2702ext[A] e q2702ext[C].
+7. Decida se a evidência comprova, de forma suficiente, perfis profissionais definidos para colaboradores de TIC/SI.
+Ao aplicar o checklist, considere a evidência como um target binário para a regra de identificação da situação encontrada. O resultado "Não conforme" será usado pela matriz como indicativo de evidência inexistente, incompatível ou insuficiente para comprovar a prática avaliada.
+Contrato de saída obrigatório:
+Responda exclusivamente em JSON válido, sem texto fora do JSON, com os campos:
+{
+  "id_avaliacao": "Q3-S3.4-q2702evi",
+  "resultado": "Conforme" ou "Não conforme",
+  "justificativa_sintetica": "&lt;fundamento objetivo da decisão&gt;",
+  "elementos_comprovados": ["&lt;elementos relevantes comprovados&gt;"],
+  "lacunas": ["&lt;elementos obrigatórios ausentes ou insuficientes&gt;"],
+  "inconsistencias": ["&lt;incompatibilidades entre evidência, resposta declarada ou escopo&gt;"]
+}
+Regra de decisão binária:
+- Retorne "Conforme" somente quando a evidência for existente, compatível e suficiente para comprovar todos os elementos essenciais da avaliação descrita.
+- Retorne "Não conforme" quando a evidência for inexistente, ilegível, incompatível, desatualizada, meramente declaratória sem comprovação documental suficiente, ou quando faltar qualquer elemento essencial da avaliação.
+- Não use classificações intermediárias, como parcialmente conforme, parcialmente suficiente ou inconclusivo. Em caso de dúvida relevante, retorne "Não conforme" e descreva a lacuna.
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="210" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Q3-S3.4-q2704evi</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Q3 - Capacidade Institucional de TIC e Segurança da Informação</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>S3.4 - Perfis profissionais de TIC e segurança da informação inexistentes, insuficientes ou não utilizados na escolha de gestores.</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>q2704evi</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Verificar se a evidência comprova que a escolha de gestores de TIC/SI utiliza perfis profissionais previamente definidos.</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Você é avaliador de evidências da Fiscalização TCE-RJ nº 18/2026 - iGovTI 2026. Analise exclusivamente a evidência anexada ao item indicado. Não busque informações externas, não presuma fatos não documentados e não utilize conhecimento fora da evidência fornecida.
+ID da avaliação: Q3-S3.4-q2704evi.
+Objetivo da avaliação: verificar se a evidência comprova que a escolha de gestores de TIC e segurança da informação ocorre segundo perfis profissionais previamente definidos e documentados.
+Contexto da situação encontrada: S3.4 - Perfis profissionais de TIC e segurança da informação inexistentes, insuficientes ou não utilizados na escolha de gestores.
+Item de evidência avaliado: q2704evi.
+Evidência esperada no questionário: perfis profissionais documentados; critérios de seleção; registros de avaliação prévia de impedimentos legais; utilização de entrevistas, análises curriculares ou outras ferramentas estruturadas; currículos publicados; atos de designação; ou outras evidências cabíveis, indicando a abrangência na organização.
+Critérios da matriz aplicáveis: C1 - COBIT 2019 APO01.05; C2 - COBIT 2019 APO07.01; C4 - COBIT 2019 APO07.03; C9 - ABNT NBR ISO/IEC 27001:2022, cláusulas 5.3 e 7.2.
+Checklist obrigatório:
+1. Identifique o tipo documental apresentado e se ele possui caráter formal ou institucional.
+2. Verifique se há perfis profissionais previamente definidos para os cargos ou funções de gestão avaliados.
+3. Verifique se a escolha ou designação de gestores considera perfil profissional, competências, experiência ou requisitos documentados.
+4. Verifique se há registros de aplicação do critério, como avaliação curricular, ferramenta estruturada, justificativa de designação ou ato formal.
+5. Verifique se a evidência permite vincular o gestor ou função avaliada à organização auditada.
+6. Verifique se a evidência é compatível com a resposta declarada em q2704ext[B].
+7. Decida se a evidência comprova, de forma suficiente, o uso de perfis previamente definidos na escolha de gestores de TIC/SI.
+Ao aplicar o checklist, considere a evidência como um target binário para a regra de identificação da situação encontrada. O resultado "Não conforme" será usado pela matriz como indicativo de evidência inexistente, incompatível ou insuficiente para comprovar a prática avaliada.
+Contrato de saída obrigatório:
+Responda exclusivamente em JSON válido, sem texto fora do JSON, com os campos:
+{
+  "id_avaliacao": "Q3-S3.4-q2704evi",
+  "resultado": "Conforme" ou "Não conforme",
+  "justificativa_sintetica": "&lt;fundamento objetivo da decisão&gt;",
+  "elementos_comprovados": ["&lt;elementos relevantes comprovados&gt;"],
+  "lacunas": ["&lt;elementos obrigatórios ausentes ou insuficientes&gt;"],
+  "inconsistencias": ["&lt;incompatibilidades entre evidência, resposta declarada ou escopo&gt;"]
+}
+Regra de decisão binária:
+- Retorne "Conforme" somente quando a evidência for existente, compatível e suficiente para comprovar todos os elementos essenciais da avaliação descrita.
+- Retorne "Não conforme" quando a evidência for inexistente, ilegível, incompatível, desatualizada, meramente declaratória sem comprovação documental suficiente, ou quando faltar qualquer elemento essencial da avaliação.
+- Não use classificações intermediárias, como parcialmente conforme, parcialmente suficiente ou inconclusivo. Em caso de dúvida relevante, retorne "Não conforme" e descreva a lacuna.
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="210" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Q3-S3.5-q2705evi</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Q3 - Capacidade Institucional de TIC e Segurança da Informação</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>S3.5 - Lacunas de competências dos colaboradores e gestores de TIC e segurança da informação não são identificadas ou tratadas.</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>q2705evi</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Verificar se a evidência comprova identificação documentada de lacunas de competências de gestores, colaboradores de TIC e segurança da informação.</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Você é avaliador de evidências da Fiscalização TCE-RJ nº 18/2026 - iGovTI 2026. Analise exclusivamente a evidência anexada ao item indicado. Não busque informações externas, não presuma fatos não documentados e não utilize conhecimento fora da evidência fornecida.
+ID da avaliação: Q3-S3.5-q2705evi.
+Objetivo da avaliação: verificar se a evidência comprova identificação documentada de lacunas de competências de gestores, colaboradores de TIC e segurança da informação.
+Contexto da situação encontrada: S3.5 - Lacunas de competências dos colaboradores e gestores de TIC e segurança da informação não são identificadas ou tratadas.
+Item de evidência avaliado: q2705evi.
+Evidência esperada no questionário: matrizes de competências; avaliações de perfil; levantamentos de necessidades de capacitação; diagnósticos de competências técnicas e gerenciais; planos de desenvolvimento; relatórios ou registros documentados; ou outras evidências cabíveis, indicando a abrangência na organização.
+Critérios da matriz aplicáveis: C4 - COBIT 2019 APO07.03; C9 - ABNT NBR ISO/IEC 27001:2022, cláusula 7.2; C10 - ABNT NBR ISO/IEC 27002:2022, controle 6.3.
+Checklist obrigatório:
+1. Identifique o tipo documental apresentado e se ele possui caráter formal, técnico ou institucional.
+2. Verifique se a evidência identifica lacunas de competências de liderança, gestão, TIC ou segurança da informação.
+3. Verifique se o diagnóstico contempla colaboradores e/ou gestores compatíveis com o escopo declarado pela organização.
+4. Verifique se há método, matriz, levantamento, avaliação ou critério documentado para identificar as lacunas.
+5. Verifique se a evidência indica data, período, responsáveis ou abrangência suficiente para demonstrar uso institucional.
+6. Verifique se a evidência é compatível com as respostas declaradas em q2705ext[B], q2705ext[C] e q2705ext[D].
+7. Decida se a evidência comprova, de forma suficiente, a identificação documentada de lacunas de competências em TIC/SI.
+Ao aplicar o checklist, considere a evidência como um target binário para a regra de identificação da situação encontrada. O resultado "Não conforme" será usado pela matriz como indicativo de evidência inexistente, incompatível ou insuficiente para comprovar a prática avaliada.
+Contrato de saída obrigatório:
+Responda exclusivamente em JSON válido, sem texto fora do JSON, com os campos:
+{
+  "id_avaliacao": "Q3-S3.5-q2705evi",
+  "resultado": "Conforme" ou "Não conforme",
+  "justificativa_sintetica": "&lt;fundamento objetivo da decisão&gt;",
+  "elementos_comprovados": ["&lt;elementos relevantes comprovados&gt;"],
+  "lacunas": ["&lt;elementos obrigatórios ausentes ou insuficientes&gt;"],
+  "inconsistencias": ["&lt;incompatibilidades entre evidência, resposta declarada ou escopo&gt;"]
+}
+Regra de decisão binária:
+- Retorne "Conforme" somente quando a evidência for existente, compatível e suficiente para comprovar todos os elementos essenciais da avaliação descrita.
+- Retorne "Não conforme" quando a evidência for inexistente, ilegível, incompatível, desatualizada, meramente declaratória sem comprovação documental suficiente, ou quando faltar qualquer elemento essencial da avaliação.
+- Não use classificações intermediárias, como parcialmente conforme, parcialmente suficiente ou inconclusivo. Em caso de dúvida relevante, retorne "Não conforme" e descreva a lacuna.
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="210" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Q3-S3.5-q2706evi</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Q3 - Capacidade Institucional de TIC e Segurança da Informação</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>S3.5 - Lacunas de competências dos colaboradores e gestores de TIC e segurança da informação não são identificadas ou tratadas.</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>q2706evi</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Verificar se a evidência comprova tratamento das lacunas de competências em TIC e segurança da informação.</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Você é avaliador de evidências da Fiscalização TCE-RJ nº 18/2026 - iGovTI 2026. Analise exclusivamente a evidência anexada ao item indicado. Não busque informações externas, não presuma fatos não documentados e não utilize conhecimento fora da evidência fornecida.
+ID da avaliação: Q3-S3.5-q2706evi.
+Objetivo da avaliação: verificar se a evidência comprova tratamento das lacunas de competências dos colaboradores e gestores de TIC e segurança da informação.
+Contexto da situação encontrada: S3.5 - Lacunas de competências dos colaboradores e gestores de TIC e segurança da informação não são identificadas ou tratadas.
+Item de evidência avaliado: q2706evi.
+Evidência esperada no questionário: plano de capacitação ou treinamento; registros de participação em cursos e treinamentos; ações de incentivo à capacitação; acompanhamento de participação e resultados; revisões periódicas do plano de capacitação; contratações ou apoio especializado; ou outras evidências cabíveis, indicando a abrangência na organização.
+Critérios da matriz aplicáveis: C4 - COBIT 2019 APO07.03; C9 - ABNT NBR ISO/IEC 27001:2022, cláusula 7.2; C10 - ABNT NBR ISO/IEC 27002:2022, controle 6.3.
+Checklist obrigatório:
+1. Identifique o tipo documental apresentado e se ele possui caráter formal, técnico ou institucional.
+2. Verifique se a evidência apresenta plano, ações ou mecanismos de tratamento de lacunas de competências em TIC/SI.
+3. Verifique se há ações de capacitação, realocação, provimento, contratação, apoio especializado ou desenvolvimento compatíveis com as lacunas identificadas.
+4. Verifique se há incentivo, monitoramento de participação, acompanhamento de resultados ou revisão periódica do plano de capacitação.
+5. Verifique se a evidência indica data, período, responsáveis ou abrangência suficiente para demonstrar execução institucional.
+6. Verifique se a evidência é compatível com as respostas declaradas em q2706ext[A], q2706ext[B] e q2706ext[C].
+7. Decida se a evidência comprova, de forma suficiente, o tratamento das lacunas de competências em TIC/SI.
+Ao aplicar o checklist, considere a evidência como um target binário para a regra de identificação da situação encontrada. O resultado "Não conforme" será usado pela matriz como indicativo de evidência inexistente, incompatível ou insuficiente para comprovar a prática avaliada.
+Contrato de saída obrigatório:
+Responda exclusivamente em JSON válido, sem texto fora do JSON, com os campos:
+{
+  "id_avaliacao": "Q3-S3.5-q2706evi",
+  "resultado": "Conforme" ou "Não conforme",
+  "justificativa_sintetica": "&lt;fundamento objetivo da decisão&gt;",
+  "elementos_comprovados": ["&lt;elementos relevantes comprovados&gt;"],
+  "lacunas": ["&lt;elementos obrigatórios ausentes ou insuficientes&gt;"],
+  "inconsistencias": ["&lt;incompatibilidades entre evidência, resposta declarada ou escopo&gt;"]
+}
+Regra de decisão binária:
+- Retorne "Conforme" somente quando a evidência for existente, compatível e suficiente para comprovar todos os elementos essenciais da avaliação descrita.
+- Retorne "Não conforme" quando a evidência for inexistente, ilegível, incompatível, desatualizada, meramente declaratória sem comprovação documental suficiente, ou quando faltar qualquer elemento essencial da avaliação.
+- Não use classificações intermediárias, como parcialmente conforme, parcialmente suficiente ou inconclusivo. Em caso de dúvida relevante, retorne "Não conforme" e descreva a lacuna.
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="210" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Q3-S3.6-q2703evi</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Q3 - Capacidade Institucional de TIC e Segurança da Informação</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>S3.6 - Modelo de operação de TIC predominantemente terceirizado ou externo, sem capacidade interna mínima declarada para coordenação, planejamento, aprovação técnica ou fiscalização das atividades críticas de TIC.</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>q2703evi</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Verificar se a evidência de dimensionamento de pessoal demonstra capacidade interna mínima para coordenar e fiscalizar TIC em modelo terceirizado ou externo.</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Você é avaliador de evidências da Fiscalização TCE-RJ nº 18/2026 - iGovTI 2026. Analise exclusivamente a evidência anexada ao item indicado. Não busque informações externas, não presuma fatos não documentados e não utilize conhecimento fora da evidência fornecida.
+ID da avaliação: Q3-S3.6-q2703evi.
+Objetivo da avaliação: verificar se a evidência de dimensionamento de pessoal demonstra capacidade interna mínima para coordenação, planejamento, aprovação técnica e fiscalização de TIC quando houver dependência relevante de terceiros ou estrutura externa.
+Contexto da situação encontrada: S3.6 - Modelo de operação de TIC predominantemente terceirizado ou externo, sem capacidade interna mínima declarada para coordenação, planejamento, aprovação técnica ou fiscalização das atividades críticas de TIC.
+Item de evidência avaliado: q2703evi.
+Evidência esperada no questionário: política ou metodologia de dimensionamento; estudos ou relatórios técnicos; definição documentada do quantitativo necessário; critérios utilizados, como serviços, sistemas, demanda, riscos ou complexidade; revisões periódicas; planos de provimento; ou outras evidências cabíveis, indicando a abrangência na organização.
+Critérios da matriz aplicáveis: C2 - COBIT 2019 APO07.01; C5 - COBIT 2019 APO07.05; C6 - COBIT 2019 APO07.06; C8 - COBIT 2019 DSS01.02.
+Checklist obrigatório:
+1. Identifique o tipo documental apresentado e se ele possui caráter formal, técnico ou institucional.
+2. Verifique se a evidência considera a dependência de terceiros, estrutura externa, contratos ou serviços críticos de TIC no dimensionamento de pessoal.
+3. Verifique se há capacidade interna prevista para coordenação, planejamento, aprovação técnica, fiscalização contratual ou retenção de conhecimento.
+4. Verifique se o quantitativo necessário é definido com base em critérios técnicos e não apenas em quadro existente ou disponibilidade orçamentária genérica.
+5. Verifique se a evidência é compatível com o modelo declarado em q0101 e com as respostas q2703ext[B] e q2703ext[C].
+6. Verifique se a evidência reduz o risco de dependência excessiva de fornecedores ou estrutura externa sem governabilidade interna.
+7. Decida se a evidência comprova, de forma suficiente, capacidade interna mínima planejada para coordenar e fiscalizar TIC.
+Ao aplicar o checklist, considere a evidência como um target binário para a regra de identificação da situação encontrada. O resultado "Não conforme" será usado pela matriz como indicativo de evidência inexistente, incompatível ou insuficiente para comprovar a prática avaliada.
+Contrato de saída obrigatório:
+Responda exclusivamente em JSON válido, sem texto fora do JSON, com os campos:
+{
+  "id_avaliacao": "Q3-S3.6-q2703evi",
+  "resultado": "Conforme" ou "Não conforme",
+  "justificativa_sintetica": "&lt;fundamento objetivo da decisão&gt;",
+  "elementos_comprovados": ["&lt;elementos relevantes comprovados&gt;"],
+  "lacunas": ["&lt;elementos obrigatórios ausentes ou insuficientes&gt;"],
+  "inconsistencias": ["&lt;incompatibilidades entre evidência, resposta declarada ou escopo&gt;"]
+}
+Regra de decisão binária:
+- Retorne "Conforme" somente quando a evidência for existente, compatível e suficiente para comprovar todos os elementos essenciais da avaliação descrita.
+- Retorne "Não conforme" quando a evidência for inexistente, ilegível, incompatível, desatualizada, meramente declaratória sem comprovação documental suficiente, ou quando faltar qualquer elemento essencial da avaliação.
+- Não use classificações intermediárias, como parcialmente conforme, parcialmente suficiente ou inconclusivo. Em caso de dúvida relevante, retorne "Não conforme" e descreva a lacuna.
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="210" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Q3-S3.6-q2801evi</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Q3 - Capacidade Institucional de TIC e Segurança da Informação</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>S3.6 - Modelo de operação de TIC predominantemente terceirizado ou externo, sem capacidade interna mínima declarada para coordenação, planejamento, aprovação técnica ou fiscalização das atividades críticas de TIC.</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>q2801evi</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Verificar se a evidência comprova processo e artefatos de gestão e fiscalização contratual de TIC com papéis, responsabilidades e controles suficientes.</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Você é avaliador de evidências da Fiscalização TCE-RJ nº 18/2026 - iGovTI 2026. Analise exclusivamente a evidência anexada ao item indicado. Não busque informações externas, não presuma fatos não documentados e não utilize conhecimento fora da evidência fornecida.
+ID da avaliação: Q3-S3.6-q2801evi.
+Objetivo da avaliação: verificar se a evidência comprova processo e artefatos de gestão e fiscalização contratual de TIC capazes de assegurar coordenação, fiscalização e responsabilização interna sobre terceiros.
+Contexto da situação encontrada: S3.6 - Modelo de operação de TIC predominantemente terceirizado ou externo, sem capacidade interna mínima declarada para coordenação, planejamento, aprovação técnica ou fiscalização das atividades críticas de TIC.
+Item de evidência avaliado: q2801evi.
+Evidência esperada no questionário: manuais, fluxos, normas ou procedimentos internos; modelos padronizados de documentos; checklists; definição de papéis e responsabilidades; fluxogramas; instruções de trabalho; artefatos de planejamento da contratação; processos de fiscalização contratual; referências à Lei 14.133/2021 e normativos correlatos; ou outras evidências cabíveis, indicando a abrangência na organização.
+Critérios da matriz aplicáveis: C1 - COBIT 2019 APO01.05; C6 - COBIT 2019 APO07.06; C7 - COBIT 2019 APO10.04; C8 - COBIT 2019 DSS01.02.
+Checklist obrigatório:
+1. Identifique o tipo documental apresentado e se ele possui caráter formal ou institucional.
+2. Verifique se o processo de gestão e fiscalização de contratos de TIC define etapas, responsáveis, papéis e controles.
+3. Verifique se há artefatos padronizados para fiscalização, como plano de fiscalização, termos de recebimento, relatórios, registros de ocorrências ou avaliação de desempenho.
+4. Verifique se os papéis internos são suficientes para supervisionar fornecedores e preservar responsabilização da organização.
+5. Verifique se o processo contempla gestão de riscos, conformidade, desempenho ou transferência/retenção de conhecimento quando aplicável.
+6. Verifique se a evidência é compatível com as respostas declaradas em q2801ext[E] e q2801ext[F].
+7. Decida se a evidência comprova, de forma suficiente, processo e artefatos de gestão e fiscalização contratual de TIC.
+Ao aplicar o checklist, considere a evidência como um target binário para a regra de identificação da situação encontrada. O resultado "Não conforme" será usado pela matriz como indicativo de evidência inexistente, incompatível ou insuficiente para comprovar a prática avaliada.
+Contrato de saída obrigatório:
+Responda exclusivamente em JSON válido, sem texto fora do JSON, com os campos:
+{
+  "id_avaliacao": "Q3-S3.6-q2801evi",
+  "resultado": "Conforme" ou "Não conforme",
+  "justificativa_sintetica": "&lt;fundamento objetivo da decisão&gt;",
+  "elementos_comprovados": ["&lt;elementos relevantes comprovados&gt;"],
+  "lacunas": ["&lt;elementos obrigatórios ausentes ou insuficientes&gt;"],
+  "inconsistencias": ["&lt;incompatibilidades entre evidência, resposta declarada ou escopo&gt;"]
+}
+Regra de decisão binária:
+- Retorne "Conforme" somente quando a evidência for existente, compatível e suficiente para comprovar todos os elementos essenciais da avaliação descrita.
+- Retorne "Não conforme" quando a evidência for inexistente, ilegível, incompatível, desatualizada, meramente declaratória sem comprovação documental suficiente, ou quando faltar qualquer elemento essencial da avaliação.
+- Não use classificações intermediárias, como parcialmente conforme, parcialmente suficiente ou inconclusivo. Em caso de dúvida relevante, retorne "Não conforme" e descreva a lacuna.
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="210" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Q3-S3.6-q2804eviA</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Q3 - Capacidade Institucional de TIC e Segurança da Informação</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>S3.6 - Modelo de operação de TIC predominantemente terceirizado ou externo, sem capacidade interna mínima declarada para coordenação, planejamento, aprovação técnica ou fiscalização das atividades críticas de TIC.</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>q2804eviA</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Verificar se a evidência comprova aprovação técnica da área de TIC em norma regulamentadora e em caso concreto de contratação.</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Você é avaliador de evidências da Fiscalização TCE-RJ nº 18/2026 - iGovTI 2026. Analise exclusivamente a evidência anexada ao item indicado. Não busque informações externas, não presuma fatos não documentados e não utilize conhecimento fora da evidência fornecida.
+ID da avaliação: Q3-S3.6-q2804eviA.
+Objetivo da avaliação: verificar se a evidência comprova que contratações de soluções de TIC são submetidas à análise prévia e aprovação técnica da área de gestão de TIC, com norma regulamentadora e caso concreto.
+Contexto da situação encontrada: S3.6 - Modelo de operação de TIC predominantemente terceirizado ou externo, sem capacidade interna mínima declarada para coordenação, planejamento, aprovação técnica ou fiscalização das atividades críticas de TIC.
+Item de evidência avaliado: q2804eviA.
+Evidência esperada no questionário: norma regulamentando o processo de análise prévia e aprovação técnica da área de gestão de TIC e evidência de um caso concreto de contratação em que essa aprovação tenha ocorrido.
+Critérios da matriz aplicáveis: C1 - COBIT 2019 APO01.05; C6 - COBIT 2019 APO07.06; C7 - COBIT 2019 APO10.04; C8 - COBIT 2019 DSS01.02.
+Checklist obrigatório:
+1. Identifique o tipo documental apresentado e se ele possui caráter formal ou institucional.
+2. Verifique se há norma, fluxo, procedimento ou instrumento equivalente que exija análise prévia e aprovação técnica pela área de TIC.
+3. Verifique se há evidência de caso concreto em que a área de TIC realizou análise ou aprovação técnica de contratação de solução de TIC.
+4. Verifique se a aprovação técnica é atribuída à área de gestão de TIC ou responsável técnico interno, e não apenas ao fornecedor ou área demandante.
+5. Verifique se a evidência permite vincular a contratação e a aprovação técnica à organização auditada.
+6. Verifique se a evidência é compatível com a resposta declarada em q2804[A].
+7. Decida se a evidência comprova, de forma suficiente, aprovação técnica interna de TIC em norma e em caso concreto.
+Ao aplicar o checklist, considere a evidência como um target binário para a regra de identificação da situação encontrada. O resultado "Não conforme" será usado pela matriz como indicativo de evidência inexistente, incompatível ou insuficiente para comprovar a prática avaliada.
+Contrato de saída obrigatório:
+Responda exclusivamente em JSON válido, sem texto fora do JSON, com os campos:
+{
+  "id_avaliacao": "Q3-S3.6-q2804eviA",
+  "resultado": "Conforme" ou "Não conforme",
+  "justificativa_sintetica": "&lt;fundamento objetivo da decisão&gt;",
+  "elementos_comprovados": ["&lt;elementos relevantes comprovados&gt;"],
+  "lacunas": ["&lt;elementos obrigatórios ausentes ou insuficientes&gt;"],
+  "inconsistencias": ["&lt;incompatibilidades entre evidência, resposta declarada ou escopo&gt;"]
+}
+Regra de decisão binária:
+- Retorne "Conforme" somente quando a evidência for existente, compatível e suficiente para comprovar todos os elementos essenciais da avaliação descrita.
+- Retorne "Não conforme" quando a evidência for inexistente, ilegível, incompatível, desatualizada, meramente declaratória sem comprovação documental suficiente, ou quando faltar qualquer elemento essencial da avaliação.
+- Não use classificações intermediárias, como parcialmente conforme, parcialmente suficiente ou inconclusivo. Em caso de dúvida relevante, retorne "Não conforme" e descreva a lacuna.
+</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F10"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="58" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="70" customWidth="1" min="5" max="5"/>
+    <col width="120" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>id_avaliacao</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>questao_auditoria</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>situacao_encontrada</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>item_evidencia</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>descricao_avaliacao</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>prompt_checklist</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="110" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Q4-S4.1-q2201evi</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Q4 - Gest?o de Servi?os de TIC</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>S4.1 - Inexist?ncia, desatualiza??o, indisponibilidade ou insufici?ncia do cat?logo de servi?os de TIC</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>q2201evi</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Verificar se a evid?ncia comprova cat?logo de servi?os de TIC vigente, atualizado, acess?vel e aderente aos servi?os efetivamente prestados.</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Voc? deve avaliar exclusivamente a evid?ncia anexada ao item q2201evi do question?rio iGovTI 2026, sem buscar informa??es externas e sem presumir fatos n?o comprovados.
+Quest?o de auditoria: Q4 - Gest?o de Servi?os de TIC.
+Situa??o encontrada avaliada: S4.1 - Inexist?ncia, desatualiza??o, indisponibilidade ou insufici?ncia do cat?logo de servi?os de TIC.
+Item de evid?ncia: q2201evi.
+Evid?ncia esperada no question?rio: evid?ncia do cat?logo e da gest?o de n?veis de servi?o, como cat?logo de servi?os vigente, ANS firmados, defini??o de metas, registros de monitoramento, relat?rios de desempenho, canais de atendimento definidos ou evid?ncias equivalentes, indicando a abrang?ncia na organiza??o.
+Crit?rios aplic?veis da matriz: C1 - ITIL 4, gerenciamento do cat?logo de servi?os; C2 - COBIT 2019, APO09.02, catalogar servi?os facilitados por TI.
+Checklist objetivo:
+1. Verificar se h? cat?logo de servi?os de TIC em documento, portal, sistema ou instrumento equivalente.
+2. Verificar se o cat?logo identifica servi?os efetivamente prestados pela ?rea de TIC e n?o apenas uma lista gen?rica de atividades.
+3. Verificar se o cat?logo cont?m informa??es m?nimas para solicita??o ou uso dos servi?os, como descri??o, p?blico-alvo, canal de atendimento, ponto de contato, prazo, hor?rio de suporte ou meta aplic?vel.
+4. Verificar se h? indica??o de atualiza??o, vig?ncia ou compatibilidade com os servi?os e acordos de n?vel de servi?o declarados.
+5. Verificar se a evid?ncia demonstra disponibilidade ou acessibilidade do cat?logo aos usu?rios, ?reas demandantes ou equipes de suporte.
+Retorne exclusivamente um JSON v?lido, sem coment?rios fora do JSON, com as chaves: "id_avaliacao", "resultado", "justificativa_sintetica", "elementos_comprovados", "lacunas" e "inconsistencias". O campo "resultado" deve ser exatamente "Conforme" ou "N?o conforme". Use "Conforme" somente quando a evid?ncia for existente, leg?vel, compat?vel, atualizada e suficiente para todos os elementos essenciais. Use "N?o conforme" quando a evid?ncia for inexistente, ileg?vel, incompat?vel, desatualizada, meramente declarat?ria sem comprova??o suficiente, ou quando faltar qualquer elemento essencial. N?o use classifica??es intermedi?rias como parcialmente conforme, parcialmente suficiente ou inconclusivo.
+O campo "id_avaliacao" deve ser "Q4-S4.1-q2201evi".</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="110" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Q4-S4.2-q2201evi</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Q4 - Gest?o de Servi?os de TIC</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>S4.2 - Inexist?ncia de ANS, metas m?nimas ou monitoramento de n?veis de servi?o para os principais servi?os de TIC</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>q2201evi</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Verificar se a evid?ncia comprova ANS, metas m?nimas e monitoramento de n?veis de servi?o para os principais servi?os de TIC.</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Voc? deve avaliar exclusivamente a evid?ncia anexada ao item q2201evi do question?rio iGovTI 2026, sem buscar informa??es externas e sem presumir fatos n?o comprovados.
+Quest?o de auditoria: Q4 - Gest?o de Servi?os de TIC.
+Situa??o encontrada avaliada: S4.2 - Inexist?ncia de ANS, metas m?nimas ou monitoramento de n?veis de servi?o para os principais servi?os de TIC.
+Item de evid?ncia: q2201evi.
+Evid?ncia esperada no question?rio: evid?ncia do cat?logo e da gest?o de n?veis de servi?o, como cat?logo de servi?os vigente, ANS firmados, defini??o de metas, registros de monitoramento, relat?rios de desempenho, canais de atendimento definidos ou evid?ncias equivalentes, indicando a abrang?ncia na organiza??o.
+Crit?rios aplic?veis da matriz: C2 - COBIT 2019, APO09.02, catalogar servi?os facilitados por TI; C3 - ITIL 4, gerenciamento de n?vel de servi?o.
+Checklist objetivo:
+1. Verificar se h? ANS, metas m?nimas, indicadores ou par?metros objetivos de atendimento para servi?os de TIC relevantes.
+2. Verificar se os n?veis de servi?o ou metas est?o associados a servi?os identific?veis e a ?reas usu?rias ou clientes internos.
+3. Verificar se h? registros de monitoramento peri?dico, relat?rios, pain?is, atas ou evid?ncias equivalentes sobre cumprimento dos n?veis de servi?o.
+4. Verificar se a evid?ncia permite identificar resultados, desvios, descumprimentos ou medidas de acompanhamento.
+5. Verificar se a evid?ncia ? compat?vel com a resposta declarat?ria e demonstra abrang?ncia suficiente na organiza??o.
+Retorne exclusivamente um JSON v?lido, sem coment?rios fora do JSON, com as chaves: "id_avaliacao", "resultado", "justificativa_sintetica", "elementos_comprovados", "lacunas" e "inconsistencias". O campo "resultado" deve ser exatamente "Conforme" ou "N?o conforme". Use "Conforme" somente quando a evid?ncia for existente, leg?vel, compat?vel, atualizada e suficiente para todos os elementos essenciais. Use "N?o conforme" quando a evid?ncia for inexistente, ileg?vel, incompat?vel, desatualizada, meramente declarat?ria sem comprova??o suficiente, ou quando faltar qualquer elemento essencial. N?o use classifica??es intermedi?rias como parcialmente conforme, parcialmente suficiente ou inconclusivo.
+O campo "id_avaliacao" deve ser "Q4-S4.2-q2201evi".</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="110" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Q4-S4.3-q2203evi</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Q4 - Gest?o de Servi?os de TIC</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>S4.3 - Inexist?ncia ou fragilidade do invent?rio de ativos de TIC</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>q2203evi</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Verificar se a evid?ncia comprova invent?rio atualizado de ativos e servi?os de TI no contexto da gest?o de configura??o e ativos.</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Voc? deve avaliar exclusivamente a evid?ncia anexada ao item q2203evi do question?rio iGovTI 2026, sem buscar informa??es externas e sem presumir fatos n?o comprovados.
+Quest?o de auditoria: Q4 - Gest?o de Servi?os de TIC.
+Situa??o encontrada avaliada: S4.3 - Inexist?ncia ou fragilidade do invent?rio de ativos de TIC.
+Item de evid?ncia: q2203evi.
+Evid?ncia esperada no question?rio: evid?ncia da gest?o de configura??o e ativos, como invent?rio atualizado de ativos e servi?os de TI, CMDB ou base equivalente, relacionamentos entre sistemas, infraestrutura e servi?os, uso dessas informa??es em mudan?as, norma ou procedimento formal, relat?rios ou ferramentas de controle.
+Crit?rios aplic?veis da matriz: C4 - ITIL 4, gerenciamento de ativos de TI; C5 - ITIL 4, gerenciamento de configura??o de servi?o.
+Checklist objetivo:
+1. Verificar se h? invent?rio ou base consolidada de ativos de TIC, servi?os de TI ou itens de configura??o relevantes.
+2. Verificar se o invent?rio cont?m elementos m?nimos como identifica??o do ativo, tipo, servi?o relacionado, respons?vel, localiza??o, ambiente, sistema, software, equipamento ou componente de infraestrutura.
+3. Verificar se a evid?ncia indica atualiza??o, manuten??o peri?dica ou uso operacional da base.
+4. Verificar se a evid?ncia demonstra relacionamento entre ativos, sistemas, infraestrutura e servi?os, quando aplic?vel.
+5. Verificar se a abrang?ncia ? suficiente para os principais servi?os ou ativos de TIC da organiza??o.
+Retorne exclusivamente um JSON v?lido, sem coment?rios fora do JSON, com as chaves: "id_avaliacao", "resultado", "justificativa_sintetica", "elementos_comprovados", "lacunas" e "inconsistencias". O campo "resultado" deve ser exatamente "Conforme" ou "N?o conforme". Use "Conforme" somente quando a evid?ncia for existente, leg?vel, compat?vel, atualizada e suficiente para todos os elementos essenciais. Use "N?o conforme" quando a evid?ncia for inexistente, ileg?vel, incompat?vel, desatualizada, meramente declarat?ria sem comprova??o suficiente, ou quando faltar qualquer elemento essencial. N?o use classifica??es intermedi?rias como parcialmente conforme, parcialmente suficiente ou inconclusivo.
+O campo "id_avaliacao" deve ser "Q4-S4.3-q2203evi".</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="110" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Q4-S4.3-q2501evi</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Q4 - Gest?o de Servi?os de TIC</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>S4.3 - Inexist?ncia ou fragilidade do invent?rio de ativos de TIC</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>q2501evi</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Verificar se a evid?ncia comprova invent?rio de ativos associados ? informa??o e defini??o de respons?veis por ativos relevantes.</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Voc? deve avaliar exclusivamente a evid?ncia anexada ao item q2501evi do question?rio iGovTI 2026, sem buscar informa??es externas e sem presumir fatos n?o comprovados.
+Quest?o de auditoria: Q4 - Gest?o de Servi?os de TIC.
+Situa??o encontrada avaliada: S4.3 - Inexist?ncia ou fragilidade do invent?rio de ativos de TIC.
+Item de evid?ncia: q2501evi.
+Evid?ncia esperada no question?rio: evid?ncia da gest?o de ativos associados ? informa??o, como invent?rio de ativos e informa??es cr?ticas, defini??o formal de respons?veis, identifica??o de informa??es cr?ticas, controles de prote??o, norma ou procedimento formal e relat?rios de acompanhamento.
+Crit?rios aplic?veis da matriz: C4 - ITIL 4, gerenciamento de ativos de TI.
+Checklist objetivo:
+1. Verificar se h? invent?rio de ativos associados ? informa??o, tais como sistemas, bases de dados, documentos digitais, backups, equipamentos ou outros ativos que armazenem, processem ou transmitam informa??es.
+2. Verificar se o invent?rio identifica ativos ou informa??es cr?ticas, sens?veis ou relevantes para os servi?os da organiza??o.
+3. Verificar se h? respons?veis formalmente definidos pelos ativos ou pelo processo de gest?o dos ativos.
+4. Verificar se a evid?ncia indica atualiza??o, revis?o ou acompanhamento do invent?rio.
+5. Verificar se a evid?ncia ? documental e suficiente, e n?o apenas declara??o gen?rica de que o processo existe.
+Retorne exclusivamente um JSON v?lido, sem coment?rios fora do JSON, com as chaves: "id_avaliacao", "resultado", "justificativa_sintetica", "elementos_comprovados", "lacunas" e "inconsistencias". O campo "resultado" deve ser exatamente "Conforme" ou "N?o conforme". Use "Conforme" somente quando a evid?ncia for existente, leg?vel, compat?vel, atualizada e suficiente para todos os elementos essenciais. Use "N?o conforme" quando a evid?ncia for inexistente, ileg?vel, incompat?vel, desatualizada, meramente declarat?ria sem comprova??o suficiente, ou quando faltar qualquer elemento essencial. N?o use classifica??es intermedi?rias como parcialmente conforme, parcialmente suficiente ou inconclusivo.
+O campo "id_avaliacao" deve ser "Q4-S4.3-q2501evi".</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="110" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Q4-S4.3-q2504evi</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Q4 - Gest?o de Servi?os de TIC</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>S4.3 - Inexist?ncia ou fragilidade do invent?rio de ativos de TIC</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>q2504evi</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Verificar se a evid?ncia comprova invent?rio e controle de dispositivos e softwares conectados ? rede ou usados nos servi?os de TIC.</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Voc? deve avaliar exclusivamente a evid?ncia anexada ao item q2504evi do question?rio iGovTI 2026, sem buscar informa??es externas e sem presumir fatos n?o comprovados.
+Quest?o de auditoria: Q4 - Gest?o de Servi?os de TIC.
+Situa??o encontrada avaliada: S4.3 - Inexist?ncia ou fragilidade do invent?rio de ativos de TIC.
+Item de evid?ncia: q2504evi.
+Evid?ncia esperada no question?rio: evid?ncia da gest?o da seguran?a dos recursos de processamento da informa??o, incluindo invent?rio de dispositivos e softwares, registros de controle, relat?rios, ferramentas ou outros documentos que demonstrem abrang?ncia na organiza??o.
+Crit?rios aplic?veis da matriz: C4 - ITIL 4, gerenciamento de ativos de TI.
+Checklist objetivo:
+1. Verificar se h? invent?rio ou controle de dispositivos conectados ? rede, equipamentos, servidores, esta??es, recursos de nuvem ou componentes equivalentes.
+2. Verificar se h? invent?rio ou controle de softwares instalados, aplica??es, licen?as ou sistemas relevantes.
+3. Verificar se a evid?ncia cont?m dados suficientes para identifica??o, controle e atualiza??o dos ativos.
+4. Verificar se a evid?ncia demonstra abrang?ncia compat?vel com os principais ambientes ou servi?os de TIC.
+5. Desconsiderar controles de seguran?a n?o relacionados ao invent?rio quando eles n?o comprovarem identifica??o e controle de ativos.
+Retorne exclusivamente um JSON v?lido, sem coment?rios fora do JSON, com as chaves: "id_avaliacao", "resultado", "justificativa_sintetica", "elementos_comprovados", "lacunas" e "inconsistencias". O campo "resultado" deve ser exatamente "Conforme" ou "N?o conforme". Use "Conforme" somente quando a evid?ncia for existente, leg?vel, compat?vel, atualizada e suficiente para todos os elementos essenciais. Use "N?o conforme" quando a evid?ncia for inexistente, ileg?vel, incompat?vel, desatualizada, meramente declarat?ria sem comprova??o suficiente, ou quando faltar qualquer elemento essencial. N?o use classifica??es intermedi?rias como parcialmente conforme, parcialmente suficiente ou inconclusivo.
+O campo "id_avaliacao" deve ser "Q4-S4.3-q2504evi".</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="110" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Q4-S4.4-q2203evi</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Q4 - Gest?o de Servi?os de TIC</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>S4.4 - Aus?ncia ou fragilidade do processo de gest?o de configura??o</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>q2203evi</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Verificar se a evid?ncia comprova processo formal ou mecanismo equivalente de gest?o de configura??o e seus relacionamentos.</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Voc? deve avaliar exclusivamente a evid?ncia anexada ao item q2203evi do question?rio iGovTI 2026, sem buscar informa??es externas e sem presumir fatos n?o comprovados.
+Quest?o de auditoria: Q4 - Gest?o de Servi?os de TIC.
+Situa??o encontrada avaliada: S4.4 - Aus?ncia ou fragilidade do processo de gest?o de configura??o.
+Item de evid?ncia: q2203evi.
+Evid?ncia esperada no question?rio: evid?ncia da gest?o de configura??o e ativos, como invent?rio atualizado de ativos e servi?os de TI, CMDB ou base equivalente, relacionamentos entre sistemas, infraestrutura e servi?os, uso dessas informa??es em mudan?as, norma ou procedimento formal, relat?rios ou ferramentas de controle.
+Crit?rios aplic?veis da matriz: C5 - ITIL 4, gerenciamento de configura??o de servi?o; C6 - COBIT 2019, BAI10.01, estabelecer e manter modelo de configura??o.
+Checklist objetivo:
+1. Verificar se h? norma, procedimento, guia, fluxo, pol?tica, ferramenta ou mecanismo equivalente para gest?o de configura??o.
+2. Verificar se a evid?ncia define ou demonstra itens de configura??o, atributos m?nimos, relacionamentos e respons?veis.
+3. Verificar se h? CMDB, base de configura??o, invent?rio estruturado ou ferramenta equivalente mantida pela organiza??o.
+4. Verificar se a base de configura??o ? usada ou referenciada em mudan?as, opera??o, an?lise de impacto ou gest?o dos servi?os.
+5. Verificar se a evid?ncia ? suficiente para comprovar processo executado ou mecanismo operacional, e n?o apenas inten??o futura.
+Retorne exclusivamente um JSON v?lido, sem coment?rios fora do JSON, com as chaves: "id_avaliacao", "resultado", "justificativa_sintetica", "elementos_comprovados", "lacunas" e "inconsistencias". O campo "resultado" deve ser exatamente "Conforme" ou "N?o conforme". Use "Conforme" somente quando a evid?ncia for existente, leg?vel, compat?vel, atualizada e suficiente para todos os elementos essenciais. Use "N?o conforme" quando a evid?ncia for inexistente, ileg?vel, incompat?vel, desatualizada, meramente declarat?ria sem comprova??o suficiente, ou quando faltar qualquer elemento essencial. N?o use classifica??es intermedi?rias como parcialmente conforme, parcialmente suficiente ou inconclusivo.
+O campo "id_avaliacao" deve ser "Q4-S4.4-q2203evi".</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="110" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Q4-S4.5-q2204evi</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Q4 - Gest?o de Servi?os de TIC</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>S4.5 - Inexist?ncia ou fragilidade do processo de gest?o de incidentes de TIC</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>q2204evi</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Verificar se a evid?ncia comprova processo formal, registros rastre?veis e tratamento estruturado de incidentes de servi?os e de seguran?a da informa??o.</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Voc? deve avaliar exclusivamente a evid?ncia anexada ao item q2204evi do question?rio iGovTI 2026, sem buscar informa??es externas e sem presumir fatos n?o comprovados.
+Quest?o de auditoria: Q4 - Gest?o de Servi?os de TIC.
+Situa??o encontrada avaliada: S4.5 - Inexist?ncia ou fragilidade do processo de gest?o de incidentes de TIC.
+Item de evid?ncia: q2204evi.
+Evid?ncia esperada no question?rio: evid?ncia da gest?o de incidentes, como norma ou procedimento formal, registros de incidentes, chamados ou tickets, crit?rios de prioriza??o e escalonamento, base de conhecimento, relat?rios de atendimento, tratamento de incidentes de seguran?a, an?lise de causa raiz e a??es corretivas.
+Crit?rios aplic?veis da matriz: C7 - ITIL 4, gerenciamento de incidentes; C8 - COBIT 2019, DSS02.02, DSS02.04 e DSS02.07, requisi??es de servi?o e incidentes gerenciados.
+Checklist objetivo:
+1. Verificar se h? norma, procedimento, fluxo ou instrumento equivalente que formalize pap?is, responsabilidades, prioriza??o e escalamento de incidentes.
+2. Verificar se existem registros rastre?veis de incidentes, chamados, tickets, hist?rico de atendimento, respons?veis, datas, status e solu??o aplicada.
+3. Verificar se a resolu??o dos incidentes considera n?veis de servi?o, criticidade, impacto ou crit?rios objetivos de atendimento.
+4. Verificar se h? tratamento de incidentes de seguran?a da informa??o, com notifica??o, resposta, comunica??o ou responsabilidades definidas.
+5. Verificar se h? an?lise posterior de incidentes relevantes ou recorrentes, causa raiz, base de conhecimento, a??es corretivas ou evid?ncias equivalentes.
+Retorne exclusivamente um JSON v?lido, sem coment?rios fora do JSON, com as chaves: "id_avaliacao", "resultado", "justificativa_sintetica", "elementos_comprovados", "lacunas" e "inconsistencias". O campo "resultado" deve ser exatamente "Conforme" ou "N?o conforme". Use "Conforme" somente quando a evid?ncia for existente, leg?vel, compat?vel, atualizada e suficiente para todos os elementos essenciais. Use "N?o conforme" quando a evid?ncia for inexistente, ileg?vel, incompat?vel, desatualizada, meramente declarat?ria sem comprova??o suficiente, ou quando faltar qualquer elemento essencial. N?o use classifica??es intermedi?rias como parcialmente conforme, parcialmente suficiente ou inconclusivo.
+O campo "id_avaliacao" deve ser "Q4-S4.5-q2204evi".</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F8"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs: atualiza relatorios e papeis de trabalho
</commit_message>
<xml_diff>
--- a/01-Planejamento/03-Estrategia_e_Plano/04-Matriz_Planejamento/matriz_verificaca_evidencias.xlsx
+++ b/01-Planejamento/03-Estrategia_e_Plano/04-Matriz_Planejamento/matriz_verificaca_evidencias.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F38"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2466,120 +2466,6 @@
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>Q6-S6.5-q2801evi</t>
-        </is>
-      </c>
-      <c r="B37" s="2" t="inlineStr">
-        <is>
-          <t>Q6 - Contratações de TIC</t>
-        </is>
-      </c>
-      <c r="C37" s="2" t="inlineStr">
-        <is>
-          <t>S6.5 - Artefatos de planejamento das contratações de TIC sem requisitos técnicos, análise de riscos, segurança da informação, proteção de dados ou critérios objetivos de aceite.</t>
-        </is>
-      </c>
-      <c r="D37" s="2" t="inlineStr">
-        <is>
-          <t>q2801evi</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="inlineStr">
-        <is>
-          <t>Verificar se a evidência comprova artefatos de planejamento com requisitos técnicos, riscos, segurança, proteção de dados e critérios objetivos de aceite.</t>
-        </is>
-      </c>
-      <c r="F37" s="2" t="inlineStr">
-        <is>
-          <t>Você é avaliador de evidências de auditoria. Analise exclusivamente a evidência fornecida. Não busque informações externas, não presuma fatos não documentados e não utilize conhecimento fora da evidência analisada.
-Objetivo da avaliação: verificar se a evidência comprova artefatos de planejamento com requisitos técnicos, riscos, segurança, proteção de dados e critérios objetivos de aceite.
-Contexto da situação encontrada: S6.5 - Artefatos de planejamento das contratações de TIC sem requisitos técnicos, análise de riscos, segurança da informação, proteção de dados ou critérios objetivos de aceite.
-Evidência esperada no questionário: modelos padronizados de documentos, DFD, ETP, TR, Matriz de Riscos ou documentos equivalentes; manuais, fluxos, normas ou procedimentos internos; checklists; artefatos de planejamento da contratação; referências à Lei 14.133/2021 e normativos correlatos; ou outras evidências cabíveis, indicando a abrangência na organização.
-Checklist obrigatório:
-1. Verifique se a evidência contém ou referencia artefatos de planejamento de contratações de TIC, como DFD, ETP, TR, projeto básico, matriz de riscos ou checklist equivalente.
-2. Verifique se os artefatos ou modelos exigem definição de requisitos técnicos da solução de TIC.
-3. Verifique se há exigência de análise de riscos da contratação ou matriz de riscos aplicável.
-4. Verifique se há exigência de requisitos de segurança da informação e de proteção de dados pessoais quando a solução envolver tratamento de dados pessoais.
-5. Verifique se há critérios objetivos de aceite, recebimento, validação, homologação ou conformidade da solução contratada.
-6. Verifique se os artefatos são suficientemente aplicáveis às contratações de TIC e não apenas modelos genéricos sem conteúdo técnico mínimo.
-7. Decida se a evidência comprova, de forma suficiente, qualidade mínima dos artefatos de planejamento das contratações de TIC.
-Ao aplicar o checklist, considere a evidência como um target binário para a regra de identificação da situação encontrada. O resultado "Não conforme" será usado pela matriz como indicativo de evidência inexistente, incompatível ou insuficiente para comprovar a prática avaliada.
-Contrato de saída obrigatório:
-Responda exclusivamente em JSON válido, sem texto fora do JSON, com os campos:
-{
-  "resultado": "Conforme" ou "Não conforme",
-  "justificativa_sintetica": "&lt;fundamento objetivo da decisão&gt;",
-  "elementos_comprovados": ["&lt;elementos relevantes comprovados&gt;"],
-  "lacunas": ["&lt;elementos obrigatórios ausentes ou insuficientes&gt;"],
-  "inconsistencias": ["&lt;incompatibilidades entre evidência, resposta declarada ou escopo&gt;"]
-}
-Regra de decisão binária:
-- Retorne "Conforme" somente quando a evidência for existente, compatível e suficiente para comprovar todos os elementos essenciais da avaliação descrita.
-- Retorne "Não conforme" quando a evidência for inexistente, ilegível, incompatível, desatualizada, meramente declaratória sem comprovação documental suficiente, ou quando faltar qualquer elemento essencial da avaliação.
-- Não use classificações intermediárias, como parcialmente conforme, parcialmente suficiente ou inconclusivo. Em caso de dúvida relevante, retorne "Não conforme" e descreva a lacuna.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>Q6-S6.6-q2801evi</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>Q6 - Contratações de TIC</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t>S6.6 - Contratações de TIC sem níveis mínimos de serviço, métricas de desempenho ou critérios objetivos de fiscalização e recebimento.</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="inlineStr">
-        <is>
-          <t>q2801evi</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="inlineStr">
-        <is>
-          <t>Verificar se a evidência comprova previsão de NMS, métricas, critérios de fiscalização, recebimento e pagamento vinculado a resultados.</t>
-        </is>
-      </c>
-      <c r="F38" s="2" t="inlineStr">
-        <is>
-          <t>Você é avaliador de evidências de auditoria. Analise exclusivamente a evidência fornecida. Não busque informações externas, não presuma fatos não documentados e não utilize conhecimento fora da evidência analisada.
-Objetivo da avaliação: verificar se a evidência comprova previsão de NMS, métricas, critérios de fiscalização, recebimento e pagamento vinculado a resultados.
-Contexto da situação encontrada: S6.6 - Contratações de TIC sem níveis mínimos de serviço, métricas de desempenho ou critérios objetivos de fiscalização e recebimento.
-Evidência esperada no questionário: processos de fiscalização contratual; modelos de plano de fiscalização, termos de recebimento, relatórios de acompanhamento, registros de ocorrências, avaliações de desempenho contratual, manuais, normas, procedimentos internos, checklists ou artefatos padronizados relativos à gestão e fiscalização de contratos de TI; ou outras evidências cabíveis, indicando a abrangência na organização.
-Checklist obrigatório:
-1. Verifique se a evidência prevê níveis mínimos de serviço, indicadores, métricas de desempenho ou parâmetros objetivos de qualidade para contratações de TIC.
-2. Verifique se há critérios de fiscalização, acompanhamento, registro de ocorrências, avaliação de desempenho ou gestão contratual.
-3. Verifique se há modelos ou orientações para recebimento provisório, recebimento definitivo, aceite, glosa ou rejeição do objeto.
-4. Verifique se a evidência vincula, quando aplicável, pagamento, aceite ou medição à efetiva entrega de resultados ou níveis de qualidade.
-5. Verifique se os critérios são objetivos e verificáveis, e não apenas afirmações genéricas de que o contrato será fiscalizado.
-6. Verifique se a evidência é aplicável às contratações de TIC e à organização auditada.
-7. Decida se a evidência comprova, de forma suficiente, controle objetivo de desempenho, fiscalização e recebimento nas contratações de TIC.
-Ao aplicar o checklist, considere a evidência como um target binário para a regra de identificação da situação encontrada. O resultado "Não conforme" será usado pela matriz como indicativo de evidência inexistente, incompatível ou insuficiente para comprovar a prática avaliada.
-Contrato de saída obrigatório:
-Responda exclusivamente em JSON válido, sem texto fora do JSON, com os campos:
-{
-  "resultado": "Conforme" ou "Não conforme",
-  "justificativa_sintetica": "&lt;fundamento objetivo da decisão&gt;",
-  "elementos_comprovados": ["&lt;elementos relevantes comprovados&gt;"],
-  "lacunas": ["&lt;elementos obrigatórios ausentes ou insuficientes&gt;"],
-  "inconsistencias": ["&lt;incompatibilidades entre evidência, resposta declarada ou escopo&gt;"]
-}
-Regra de decisão binária:
-- Retorne "Conforme" somente quando a evidência for existente, compatível e suficiente para comprovar todos os elementos essenciais da avaliação descrita.
-- Retorne "Não conforme" quando a evidência for inexistente, ilegível, incompatível, desatualizada, meramente declaratória sem comprovação documental suficiente, ou quando faltar qualquer elemento essencial da avaliação.
-- Não use classificações intermediárias, como parcialmente conforme, parcialmente suficiente ou inconclusivo. Em caso de dúvida relevante, retorne "Não conforme" e descreva a lacuna.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <autoFilter ref="A1:F38"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>